<commit_message>
removing old data formats
</commit_message>
<xml_diff>
--- a/data/vip2026.xlsx
+++ b/data/vip2026.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="27">
   <si>
     <t>left</t>
   </si>
@@ -24,7 +24,7 @@
     <t>right</t>
   </si>
   <si>
-    <t>dm</t>
+    <t>mm</t>
   </si>
   <si>
     <t>Bennet</t>
@@ -554,105 +554,96 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="10" width="10.7109375" customWidth="1"/>
+    <col min="1" max="9" width="10.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="J1" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:10">
+    <row r="2" spans="1:9">
       <c r="A2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F2" t="s">
+        <v>22</v>
+      </c>
+      <c r="G2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" t="s">
+        <v>22</v>
+      </c>
+      <c r="G3" t="s">
+        <v>21</v>
+      </c>
+      <c r="H3" t="s">
         <v>14</v>
       </c>
-      <c r="B2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F2" t="s">
-        <v>21</v>
-      </c>
-      <c r="G2" t="s">
-        <v>22</v>
-      </c>
-      <c r="H2" t="s">
-        <v>13</v>
-      </c>
-      <c r="I2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10">
-      <c r="A3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C3" t="s">
-        <v>18</v>
-      </c>
-      <c r="D3" t="s">
-        <v>20</v>
-      </c>
-      <c r="E3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F3" t="s">
-        <v>17</v>
-      </c>
-      <c r="G3" t="s">
-        <v>22</v>
-      </c>
-      <c r="H3" t="s">
-        <v>21</v>
-      </c>
-      <c r="I3" t="s">
-        <v>14</v>
-      </c>
-      <c r="J3">
+      <c r="I3">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
cleanup and adding solution to excel files
</commit_message>
<xml_diff>
--- a/data/vip2026.xlsx
+++ b/data/vip2026.xlsx
@@ -1,22 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11102"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/isabelhaas/Documents/Coding/aytogermany/data/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC79D9DE-2771-9340-A6AD-908C60F2A25A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="17120" yWindow="5560" windowWidth="20160" windowHeight="16440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Candidates" sheetId="1" r:id="rId1"/>
     <sheet name="Nights" sheetId="2" r:id="rId2"/>
     <sheet name="Matchboxes" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="27">
   <si>
     <t>left</t>
   </si>
@@ -102,8 +108,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -120,7 +126,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -130,6 +136,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFC5C6C7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -146,24 +158,33 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -201,7 +222,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -235,6 +256,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -269,9 +291,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -444,14 +467,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C12"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="3" width="10.7109375" customWidth="1"/>
+    <col min="1" max="3" width="10.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -462,7 +485,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -470,7 +493,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -478,7 +501,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -486,7 +509,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -494,7 +517,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -502,7 +525,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -510,7 +533,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -518,7 +541,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>10</v>
       </c>
@@ -526,7 +549,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>11</v>
       </c>
@@ -534,7 +557,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>12</v>
       </c>
@@ -542,7 +565,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="12" spans="1:3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="B12" t="s">
         <v>23</v>
       </c>
@@ -553,97 +576,150 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:K4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="9" width="10.7109375" customWidth="1"/>
+    <col min="3" max="11" width="10.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" t="s">
         <v>23</v>
       </c>
-      <c r="B2" t="s">
+      <c r="D2" t="s">
         <v>20</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E2" t="s">
         <v>17</v>
       </c>
-      <c r="D2" t="s">
+      <c r="F2" t="s">
         <v>15</v>
       </c>
-      <c r="E2" t="s">
+      <c r="G2" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="F2" t="s">
+      <c r="H2" t="s">
         <v>22</v>
       </c>
-      <c r="G2" t="s">
+      <c r="I2" t="s">
         <v>13</v>
       </c>
-      <c r="H2" t="s">
+      <c r="J2" t="s">
         <v>18</v>
       </c>
-      <c r="I2">
+      <c r="K2">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" t="s">
         <v>23</v>
       </c>
-      <c r="B3" t="s">
+      <c r="D3" t="s">
         <v>18</v>
       </c>
-      <c r="C3" t="s">
+      <c r="E3" t="s">
         <v>20</v>
       </c>
-      <c r="D3" t="s">
+      <c r="F3" t="s">
         <v>15</v>
       </c>
-      <c r="E3" t="s">
+      <c r="G3" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="F3" t="s">
+      <c r="H3" t="s">
         <v>22</v>
       </c>
-      <c r="G3" t="s">
+      <c r="I3" t="s">
         <v>21</v>
       </c>
-      <c r="H3" t="s">
+      <c r="J3" t="s">
         <v>14</v>
       </c>
-      <c r="I3">
+      <c r="K3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H4" t="s">
+        <v>19</v>
+      </c>
+      <c r="I4" t="s">
+        <v>22</v>
+      </c>
+      <c r="J4" t="s">
+        <v>14</v>
+      </c>
+      <c r="K4">
         <v>3</v>
       </c>
     </row>
@@ -653,14 +729,14 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="4" width="10.7109375" customWidth="1"/>
+    <col min="1" max="4" width="10.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>25</v>
       </c>
@@ -674,7 +750,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>0</v>
       </c>
@@ -688,7 +764,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>0</v>
       </c>
@@ -702,7 +778,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>1</v>
       </c>
@@ -714,6 +790,34 @@
       </c>
       <c r="D4" t="b">
         <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>2</v>
+      </c>
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" t="s">
+        <v>21</v>
+      </c>
+      <c r="D5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>2</v>
+      </c>
+      <c r="B6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
vip2026 functionality with Laurenz
</commit_message>
<xml_diff>
--- a/data/vip2026.xlsx
+++ b/data/vip2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/isabelhaas/Documents/Coding/aytogermany/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC79D9DE-2771-9340-A6AD-908C60F2A25A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F32E29E8-6D65-744C-A0B9-4476B7C06320}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="17120" yWindow="5560" windowWidth="20160" windowHeight="16440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1560" yWindow="2540" windowWidth="28400" windowHeight="18240" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Candidates" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="28">
   <si>
     <t>left</t>
   </si>
@@ -103,6 +103,9 @@
   </si>
   <si>
     <t>result</t>
+  </si>
+  <si>
+    <t>Laurenz</t>
   </si>
 </sst>
 </file>
@@ -158,12 +161,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -566,6 +570,9 @@
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>27</v>
+      </c>
       <c r="B12" t="s">
         <v>23</v>
       </c>
@@ -619,28 +626,28 @@
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+      <c r="A2" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="3" t="s">
         <v>15</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="H2" t="s">
+      <c r="H2" s="3" t="s">
         <v>22</v>
       </c>
       <c r="I2" t="s">
@@ -654,28 +661,28 @@
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+      <c r="A3" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3" s="3" t="s">
         <v>15</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H3" t="s">
+      <c r="H3" s="3" t="s">
         <v>22</v>
       </c>
       <c r="I3" t="s">
@@ -689,22 +696,22 @@
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
+      <c r="A4" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F4" s="3" t="s">
         <v>13</v>
       </c>
       <c r="G4" s="2" t="s">

</xml_diff>

<commit_message>
file restructuring, test data & week 4
</commit_message>
<xml_diff>
--- a/data/vip2026.xlsx
+++ b/data/vip2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/isabelhaas/Documents/Coding/aytogermany/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F32E29E8-6D65-744C-A0B9-4476B7C06320}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5000BB65-21CD-694F-A7B1-9946C3728803}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1560" yWindow="2540" windowWidth="28400" windowHeight="18240" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19180" yWindow="760" windowWidth="19220" windowHeight="24100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Candidates" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="28">
   <si>
     <t>left</t>
   </si>
@@ -161,13 +161,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -584,7 +583,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="11" width="10.6640625" customWidth="1"/>
@@ -626,28 +625,28 @@
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A2" s="3" t="s">
+      <c r="A2" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" t="s">
         <v>23</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" t="s">
         <v>20</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" t="s">
         <v>17</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" t="s">
         <v>15</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="H2" t="s">
         <v>22</v>
       </c>
       <c r="I2" t="s">
@@ -661,28 +660,28 @@
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A3" s="3" t="s">
+      <c r="A3" t="s">
         <v>19</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" t="s">
         <v>23</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" t="s">
         <v>20</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" t="s">
         <v>15</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="H3" t="s">
         <v>22</v>
       </c>
       <c r="I3" t="s">
@@ -696,22 +695,22 @@
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A4" s="3" t="s">
+      <c r="A4" t="s">
         <v>20</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" t="s">
         <v>18</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" t="s">
         <v>23</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" t="s">
         <v>15</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" t="s">
         <v>13</v>
       </c>
       <c r="G4" s="2" t="s">
@@ -728,6 +727,41 @@
       </c>
       <c r="K4">
         <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E5" t="s">
+        <v>23</v>
+      </c>
+      <c r="F5" t="s">
+        <v>22</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H5" t="s">
+        <v>15</v>
+      </c>
+      <c r="I5" t="s">
+        <v>16</v>
+      </c>
+      <c r="J5" t="s">
+        <v>19</v>
+      </c>
+      <c r="K5">
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -737,7 +771,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="4" width="10.6640625" customWidth="1"/>
@@ -827,6 +861,20 @@
         <v>1</v>
       </c>
     </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
make solution frozen, refacter for solver
</commit_message>
<xml_diff>
--- a/data/vip2026.xlsx
+++ b/data/vip2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/isabelhaas/Documents/Coding/aytogermany/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5000BB65-21CD-694F-A7B1-9946C3728803}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0F996E2-0ECE-E740-B849-51E321EB2360}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19180" yWindow="760" windowWidth="19220" windowHeight="24100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11680" yWindow="1740" windowWidth="19220" windowHeight="24100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Candidates" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
fixed so that all seasons match aytorakel
</commit_message>
<xml_diff>
--- a/data/vip2026.xlsx
+++ b/data/vip2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/isabelhaas/Documents/Coding/aytogermany/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0F996E2-0ECE-E740-B849-51E321EB2360}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFF3D01A-AEF5-4847-A1F9-AFA9230FC1AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11680" yWindow="1740" windowWidth="19220" windowHeight="24100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="17160" yWindow="1000" windowWidth="22040" windowHeight="24100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Candidates" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="28">
   <si>
     <t>left</t>
   </si>
@@ -583,13 +583,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="3" max="11" width="10.6640625" customWidth="1"/>
+    <col min="3" max="12" width="10.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
@@ -618,13 +618,16 @@
         <v>11</v>
       </c>
       <c r="J1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -652,14 +655,14 @@
       <c r="I2" t="s">
         <v>13</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>18</v>
       </c>
-      <c r="K2">
+      <c r="L2">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>19</v>
       </c>
@@ -687,14 +690,14 @@
       <c r="I3" t="s">
         <v>21</v>
       </c>
-      <c r="J3" t="s">
+      <c r="K3" t="s">
         <v>14</v>
       </c>
-      <c r="K3">
+      <c r="L3">
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>20</v>
       </c>
@@ -722,14 +725,14 @@
       <c r="I4" t="s">
         <v>22</v>
       </c>
-      <c r="J4" t="s">
+      <c r="K4" t="s">
         <v>14</v>
       </c>
-      <c r="K4">
+      <c r="L4">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>14</v>
       </c>
@@ -757,11 +760,46 @@
       <c r="I5" t="s">
         <v>16</v>
       </c>
-      <c r="J5" t="s">
+      <c r="K5" t="s">
         <v>19</v>
       </c>
-      <c r="K5">
+      <c r="L5">
         <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F6" t="s">
+        <v>15</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H6" t="s">
+        <v>16</v>
+      </c>
+      <c r="I6" t="s">
+        <v>22</v>
+      </c>
+      <c r="J6" t="s">
+        <v>23</v>
+      </c>
+      <c r="K6" t="s">
+        <v>19</v>
+      </c>
+      <c r="L6">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>